<commit_message>
Added alumni, changed chico pic, added news
</commit_message>
<xml_diff>
--- a/members/members_list.xlsx
+++ b/members/members_list.xlsx
@@ -970,34 +970,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>52</v>
-      </c>
-    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E8" r:id="rId1" display="https://www.linkedin.com/in/frangones/"/>
@@ -1018,7 +992,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
@@ -1052,590 +1026,618 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>62</v>
+      <c r="A3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>56</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>73</v>
+        <v>61</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>81</v>
+        <v>71</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>91</v>
+        <v>71</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>118</v>
+        <v>108</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="D19" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="D21" s="3" t="s">
-        <v>133</v>
+        <v>125</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>136</v>
+        <v>107</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>47</v>
+        <v>132</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>117</v>
       </c>
+      <c r="D23" s="3" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>144</v>
+        <v>47</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>145</v>
+        <v>98</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>150</v>
+        <v>141</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>145</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>153</v>
+        <v>146</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>47</v>
+        <v>152</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>156</v>
+        <v>145</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>107</v>
+        <v>156</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>165</v>
+        <v>47</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>170</v>
+        <v>107</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>166</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>183</v>
+        <v>166</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>178</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B39" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C39" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D39" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E39" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G37" s="3" t="s">
+      <c r="G39" s="3" t="s">
         <v>193</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F5" r:id="rId1" display="https://twitter.com/Iam_Randheer"/>
-    <hyperlink ref="E19" r:id="rId2" display="https://www.linkedin.com/in/peilin-du-87a0bb238"/>
+    <hyperlink ref="F7" r:id="rId1" display="https://twitter.com/Iam_Randheer"/>
+    <hyperlink ref="E21" r:id="rId2" display="https://www.linkedin.com/in/peilin-du-87a0bb238"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>